<commit_message>
new corpus and y2 review and rephrased reviews
</commit_message>
<xml_diff>
--- a/data/reviews/human_reviews/human_reviews_human-y1.xlsx
+++ b/data/reviews/human_reviews/human_reviews_human-y1.xlsx
@@ -1,14 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20900" windowHeight="22260" activeTab="1"/>
+    <workbookView windowHeight="16020"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="262">
   <si>
     <t>year</t>
   </si>
@@ -976,57 +975,6 @@
     <t>The proposal addresses the critical challenge of metadata completeness and consistency in proteomics data, essential for understanding cellular mechanisms and disease processes. Integrating bioinformatics, NLP, and LLMs for automated metadata extraction is an innovative approach that promises to enhance metadata quality and usability.
 To improve accuracy and avoid hallucinations, the proposal could benefit from iterative validation steps and feedback loops, involving multiple rounds of testing with expert input. Allocating additional buffer time for these tasks would help manage unforeseen challenges and ensure higher reliability.</t>
   </si>
-  <si>
-    <t>proposal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">author </t>
-  </si>
-  <si>
-    <t>human review</t>
-  </si>
-  <si>
-    <t>GPT</t>
-  </si>
-  <si>
-    <t>Claude</t>
-  </si>
-  <si>
-    <t>Gemini</t>
-  </si>
-  <si>
-    <t>human-y1</t>
-  </si>
-  <si>
-    <r>
-      <t>5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; The proposed research is highly innovative as it aims to identify  cytokinetic bottlenecks under heat stress, which has not been  extensively studied previously. This approach could substantially  advance our understanding of plant responses to climate change,  particularly in terms of cellular and molecular adaptations. The  focus on comparing responses in heat-tolerant versus susceptible  species adds significant value to the novelty of the research.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; While the motivation for the research was a strength,  the lack of innovation in the proposed bioinformatics analysis was a  weakness--no new methodology was proposed to sort, parse, filter,  or integrate datasets. An outline of the sequence of steps for the  bioinformatics analysis would have been helpful.</t>
-    </r>
-  </si>
 </sst>
 </file>
 
@@ -1038,18 +986,10 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1535,170 +1475,164 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -1708,7 +1642,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -2065,7 +1999,7 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -2077,7 +2011,7 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
@@ -2103,13 +2037,13 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F2" t="s">
@@ -2121,7 +2055,7 @@
       <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="4" t="s">
         <v>19</v>
       </c>
       <c r="J2" t="s">
@@ -2133,7 +2067,7 @@
       <c r="L2" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="4" t="s">
         <v>21</v>
       </c>
       <c r="N2" t="s">
@@ -2147,37 +2081,37 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="4" t="s">
         <v>23</v>
       </c>
       <c r="H3">
         <v>4</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="4" t="s">
         <v>24</v>
       </c>
       <c r="J3">
         <v>5</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="M3" s="4" t="s">
         <v>26</v>
       </c>
       <c r="N3">
@@ -2191,37 +2125,37 @@
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F4">
         <v>4</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H4">
         <v>4</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="4" t="s">
         <v>29</v>
       </c>
       <c r="J4">
         <v>5</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="4" t="s">
         <v>30</v>
       </c>
       <c r="L4">
         <v>3</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="N4">
@@ -2235,13 +2169,13 @@
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D5">
         <v>4</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="4" t="s">
         <v>32</v>
       </c>
       <c r="F5">
@@ -2253,7 +2187,7 @@
       <c r="H5">
         <v>5</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="4" t="s">
         <v>34</v>
       </c>
       <c r="J5">
@@ -2265,27 +2199,27 @@
       <c r="L5">
         <v>3</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="M5" s="4" t="s">
         <v>36</v>
       </c>
       <c r="N5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" ht="409.5" spans="1:14">
+    <row r="6" ht="247" spans="1:14">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="4" t="s">
         <v>38</v>
       </c>
       <c r="F6" t="s">
@@ -2297,7 +2231,7 @@
       <c r="H6" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="4" t="s">
         <v>40</v>
       </c>
       <c r="J6" t="s">
@@ -2309,7 +2243,7 @@
       <c r="L6" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="4" t="s">
         <v>42</v>
       </c>
       <c r="N6" t="s">
@@ -2323,13 +2257,13 @@
       <c r="B7">
         <v>2</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="4" t="s">
         <v>43</v>
       </c>
       <c r="F7" t="s">
@@ -2341,7 +2275,7 @@
       <c r="H7" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="4" t="s">
         <v>45</v>
       </c>
       <c r="J7" t="s">
@@ -2353,7 +2287,7 @@
       <c r="L7" t="s">
         <v>17</v>
       </c>
-      <c r="M7" s="6" t="s">
+      <c r="M7" s="4" t="s">
         <v>47</v>
       </c>
       <c r="N7" t="s">
@@ -2367,25 +2301,25 @@
       <c r="B8">
         <v>2</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F8" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="4" t="s">
         <v>49</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="4" t="s">
         <v>50</v>
       </c>
       <c r="J8" t="s">
@@ -2397,7 +2331,7 @@
       <c r="L8" t="s">
         <v>17</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="N8" t="s">
@@ -2411,37 +2345,37 @@
       <c r="B9">
         <v>3</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="1" t="s">
         <v>53</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F9" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="4" t="s">
         <v>55</v>
       </c>
       <c r="H9" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="4" t="s">
         <v>56</v>
       </c>
       <c r="J9" t="s">
         <v>17</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="4" t="s">
         <v>57</v>
       </c>
       <c r="L9" t="s">
         <v>17</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="M9" s="4" t="s">
         <v>58</v>
       </c>
       <c r="N9" t="s">
@@ -2455,13 +2389,13 @@
       <c r="B10">
         <v>3</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>53</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="4" t="s">
         <v>59</v>
       </c>
       <c r="F10" t="s">
@@ -2473,7 +2407,7 @@
       <c r="H10" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" s="4" t="s">
         <v>61</v>
       </c>
       <c r="J10" t="s">
@@ -2485,7 +2419,7 @@
       <c r="L10" t="s">
         <v>17</v>
       </c>
-      <c r="M10" s="6" t="s">
+      <c r="M10" s="4" t="s">
         <v>63</v>
       </c>
       <c r="N10" t="s">
@@ -2493,31 +2427,31 @@
       </c>
     </row>
     <row r="11" ht="409.5" spans="1:14">
-      <c r="A11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="4">
+      <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="2">
         <v>3</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <v>3</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="F11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H11" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="4" t="s">
         <v>66</v>
       </c>
       <c r="J11" t="s">
@@ -2529,7 +2463,7 @@
       <c r="L11" t="s">
         <v>17</v>
       </c>
-      <c r="M11" s="6" t="s">
+      <c r="M11" s="4" t="s">
         <v>68</v>
       </c>
       <c r="N11" t="s">
@@ -2537,22 +2471,22 @@
       </c>
     </row>
     <row r="12" ht="409.5" spans="1:14">
-      <c r="A12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="4">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="2">
         <v>3</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="2">
         <v>4</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G12" t="s">
@@ -2561,7 +2495,7 @@
       <c r="H12" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="4" t="s">
         <v>71</v>
       </c>
       <c r="J12" t="s">
@@ -2573,7 +2507,7 @@
       <c r="L12" t="s">
         <v>17</v>
       </c>
-      <c r="M12" s="6" t="s">
+      <c r="M12" s="4" t="s">
         <v>73</v>
       </c>
       <c r="N12" t="s">
@@ -2587,13 +2521,13 @@
       <c r="B13">
         <v>4</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="4" t="s">
         <v>75</v>
       </c>
       <c r="F13" t="s">
@@ -2605,7 +2539,7 @@
       <c r="H13" t="s">
         <v>17</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="4" t="s">
         <v>77</v>
       </c>
       <c r="J13" t="s">
@@ -2617,7 +2551,7 @@
       <c r="L13" t="s">
         <v>17</v>
       </c>
-      <c r="M13" s="6" t="s">
+      <c r="M13" s="4" t="s">
         <v>79</v>
       </c>
       <c r="N13" t="s">
@@ -2631,13 +2565,13 @@
       <c r="B14">
         <v>4</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D14">
         <v>2</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="4" t="s">
         <v>80</v>
       </c>
       <c r="F14" t="s">
@@ -2649,7 +2583,7 @@
       <c r="H14" t="s">
         <v>17</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="4" t="s">
         <v>82</v>
       </c>
       <c r="J14" t="s">
@@ -2661,7 +2595,7 @@
       <c r="L14" t="s">
         <v>17</v>
       </c>
-      <c r="M14" s="6" t="s">
+      <c r="M14" s="4" t="s">
         <v>84</v>
       </c>
       <c r="N14" t="s">
@@ -2675,13 +2609,13 @@
       <c r="B15">
         <v>4</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D15">
         <v>3</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="4" t="s">
         <v>85</v>
       </c>
       <c r="F15" t="s">
@@ -2693,7 +2627,7 @@
       <c r="H15" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="I15" s="4" t="s">
         <v>87</v>
       </c>
       <c r="J15" t="s">
@@ -2705,7 +2639,7 @@
       <c r="L15" t="s">
         <v>17</v>
       </c>
-      <c r="M15" s="6" t="s">
+      <c r="M15" s="4" t="s">
         <v>89</v>
       </c>
       <c r="N15" t="s">
@@ -2719,37 +2653,37 @@
       <c r="B16">
         <v>4</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D16">
         <v>4</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="4" t="s">
         <v>90</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="G16" s="4" t="s">
         <v>91</v>
       </c>
       <c r="H16" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="I16" s="4" t="s">
         <v>92</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
       </c>
-      <c r="K16" s="6" t="s">
+      <c r="K16" s="4" t="s">
         <v>93</v>
       </c>
       <c r="L16" t="s">
         <v>17</v>
       </c>
-      <c r="M16" s="6" t="s">
+      <c r="M16" s="4" t="s">
         <v>94</v>
       </c>
       <c r="N16" t="s">
@@ -2763,13 +2697,13 @@
       <c r="B17">
         <v>5</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="4" t="s">
         <v>96</v>
       </c>
       <c r="F17" t="s">
@@ -2781,7 +2715,7 @@
       <c r="H17" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="4" t="s">
         <v>98</v>
       </c>
       <c r="J17" t="s">
@@ -2793,7 +2727,7 @@
       <c r="L17" t="s">
         <v>17</v>
       </c>
-      <c r="M17" s="6" t="s">
+      <c r="M17" s="4" t="s">
         <v>100</v>
       </c>
       <c r="N17" t="s">
@@ -2807,37 +2741,37 @@
       <c r="B18">
         <v>5</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D18">
         <v>2</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="4" t="s">
         <v>101</v>
       </c>
       <c r="F18" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="4" t="s">
         <v>102</v>
       </c>
       <c r="H18" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="I18" s="4" t="s">
         <v>103</v>
       </c>
       <c r="J18" t="s">
         <v>17</v>
       </c>
-      <c r="K18" s="6" t="s">
+      <c r="K18" s="4" t="s">
         <v>104</v>
       </c>
       <c r="L18" t="s">
         <v>17</v>
       </c>
-      <c r="M18" s="6" t="s">
+      <c r="M18" s="4" t="s">
         <v>105</v>
       </c>
       <c r="N18" t="s">
@@ -2851,13 +2785,13 @@
       <c r="B19">
         <v>5</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D19">
         <v>3</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="4" t="s">
         <v>106</v>
       </c>
       <c r="F19" t="s">
@@ -2869,7 +2803,7 @@
       <c r="H19" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="4" t="s">
         <v>108</v>
       </c>
       <c r="J19" t="s">
@@ -2881,7 +2815,7 @@
       <c r="L19" t="s">
         <v>17</v>
       </c>
-      <c r="M19" s="6" t="s">
+      <c r="M19" s="4" t="s">
         <v>110</v>
       </c>
       <c r="N19" t="s">
@@ -2895,37 +2829,37 @@
       <c r="B20">
         <v>5</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D20">
         <v>4</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="4" t="s">
         <v>111</v>
       </c>
       <c r="F20" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" s="4" t="s">
         <v>112</v>
       </c>
       <c r="H20" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="4" t="s">
         <v>113</v>
       </c>
       <c r="J20" t="s">
         <v>17</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="K20" s="4" t="s">
         <v>114</v>
       </c>
       <c r="L20" t="s">
         <v>17</v>
       </c>
-      <c r="M20" s="6" t="s">
+      <c r="M20" s="4" t="s">
         <v>115</v>
       </c>
       <c r="N20" t="s">
@@ -2939,13 +2873,13 @@
       <c r="B21">
         <v>6</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="1" t="s">
         <v>116</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="4" t="s">
         <v>117</v>
       </c>
       <c r="F21" t="s">
@@ -2957,7 +2891,7 @@
       <c r="H21" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="I21" s="4" t="s">
         <v>119</v>
       </c>
       <c r="J21" t="s">
@@ -2969,7 +2903,7 @@
       <c r="L21" t="s">
         <v>17</v>
       </c>
-      <c r="M21" s="6" t="s">
+      <c r="M21" s="4" t="s">
         <v>121</v>
       </c>
       <c r="N21" t="s">
@@ -2983,37 +2917,37 @@
       <c r="B22">
         <v>6</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="1" t="s">
         <v>116</v>
       </c>
       <c r="D22">
         <v>2</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="4" t="s">
         <v>122</v>
       </c>
       <c r="F22" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" s="4" t="s">
         <v>123</v>
       </c>
       <c r="H22" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="4" t="s">
         <v>124</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
       </c>
-      <c r="K22" s="5" t="s">
+      <c r="K22" s="3" t="s">
         <v>125</v>
       </c>
       <c r="L22" t="s">
         <v>17</v>
       </c>
-      <c r="M22" s="6" t="s">
+      <c r="M22" s="4" t="s">
         <v>126</v>
       </c>
       <c r="N22" t="s">
@@ -3027,13 +2961,13 @@
       <c r="B23">
         <v>6</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="1" t="s">
         <v>116</v>
       </c>
       <c r="D23">
         <v>3</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="4" t="s">
         <v>127</v>
       </c>
       <c r="F23" t="s">
@@ -3045,7 +2979,7 @@
       <c r="H23" t="s">
         <v>17</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="4" t="s">
         <v>129</v>
       </c>
       <c r="J23" t="s">
@@ -3057,7 +2991,7 @@
       <c r="L23" t="s">
         <v>17</v>
       </c>
-      <c r="M23" s="6" t="s">
+      <c r="M23" s="4" t="s">
         <v>131</v>
       </c>
       <c r="N23" t="s">
@@ -3071,37 +3005,37 @@
       <c r="B24">
         <v>6</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="1" t="s">
         <v>116</v>
       </c>
       <c r="D24">
         <v>4</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="4" t="s">
         <v>132</v>
       </c>
       <c r="F24" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="4" t="s">
         <v>133</v>
       </c>
       <c r="H24" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="6" t="s">
+      <c r="I24" s="4" t="s">
         <v>134</v>
       </c>
       <c r="J24" t="s">
         <v>17</v>
       </c>
-      <c r="K24" s="6" t="s">
+      <c r="K24" s="4" t="s">
         <v>135</v>
       </c>
       <c r="L24" t="s">
         <v>17</v>
       </c>
-      <c r="M24" s="6" t="s">
+      <c r="M24" s="4" t="s">
         <v>136</v>
       </c>
       <c r="N24" t="s">
@@ -3115,13 +3049,13 @@
       <c r="B25">
         <v>7</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="1" t="s">
         <v>137</v>
       </c>
       <c r="D25">
         <v>1</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F25">
@@ -3133,19 +3067,19 @@
       <c r="H25">
         <v>4</v>
       </c>
-      <c r="I25" s="6" t="s">
+      <c r="I25" s="4" t="s">
         <v>140</v>
       </c>
       <c r="J25">
         <v>5</v>
       </c>
-      <c r="K25" s="5" t="s">
+      <c r="K25" s="3" t="s">
         <v>141</v>
       </c>
       <c r="L25">
         <v>5</v>
       </c>
-      <c r="M25" s="6" t="s">
+      <c r="M25" s="4" t="s">
         <v>142</v>
       </c>
       <c r="N25">
@@ -3159,25 +3093,25 @@
       <c r="B26">
         <v>7</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1" t="s">
         <v>137</v>
       </c>
       <c r="D26">
         <v>2</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="4" t="s">
         <v>143</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="G26" s="4" t="s">
         <v>144</v>
       </c>
       <c r="H26">
         <v>2</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="I26" s="4" t="s">
         <v>145</v>
       </c>
       <c r="J26">
@@ -3189,7 +3123,7 @@
       <c r="L26">
         <v>3</v>
       </c>
-      <c r="M26" s="6" t="s">
+      <c r="M26" s="4" t="s">
         <v>147</v>
       </c>
       <c r="N26">
@@ -3203,13 +3137,13 @@
       <c r="B27">
         <v>7</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="1" t="s">
         <v>137</v>
       </c>
       <c r="D27">
         <v>3</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="4" t="s">
         <v>148</v>
       </c>
       <c r="F27" t="s">
@@ -3221,7 +3155,7 @@
       <c r="H27" t="s">
         <v>17</v>
       </c>
-      <c r="I27" s="6" t="s">
+      <c r="I27" s="4" t="s">
         <v>150</v>
       </c>
       <c r="J27" t="s">
@@ -3233,7 +3167,7 @@
       <c r="L27" t="s">
         <v>17</v>
       </c>
-      <c r="M27" s="6" t="s">
+      <c r="M27" s="4" t="s">
         <v>152</v>
       </c>
       <c r="N27" t="s">
@@ -3247,37 +3181,37 @@
       <c r="B28">
         <v>7</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="1" t="s">
         <v>137</v>
       </c>
       <c r="D28">
         <v>4</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="4" t="s">
         <v>153</v>
       </c>
       <c r="F28" t="s">
         <v>17</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G28" s="4" t="s">
         <v>154</v>
       </c>
       <c r="H28" t="s">
         <v>17</v>
       </c>
-      <c r="I28" s="6" t="s">
+      <c r="I28" s="4" t="s">
         <v>155</v>
       </c>
       <c r="J28" t="s">
         <v>17</v>
       </c>
-      <c r="K28" s="6" t="s">
+      <c r="K28" s="4" t="s">
         <v>156</v>
       </c>
       <c r="L28" t="s">
         <v>17</v>
       </c>
-      <c r="M28" s="6" t="s">
+      <c r="M28" s="4" t="s">
         <v>157</v>
       </c>
       <c r="N28" t="s">
@@ -3291,13 +3225,13 @@
       <c r="B29">
         <v>8</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="1" t="s">
         <v>158</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="4" t="s">
         <v>159</v>
       </c>
       <c r="F29" t="s">
@@ -3309,7 +3243,7 @@
       <c r="H29" t="s">
         <v>17</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I29" s="4" t="s">
         <v>161</v>
       </c>
       <c r="J29" t="s">
@@ -3321,7 +3255,7 @@
       <c r="L29" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="6" t="s">
+      <c r="M29" s="4" t="s">
         <v>163</v>
       </c>
       <c r="N29" t="s">
@@ -3335,37 +3269,37 @@
       <c r="B30">
         <v>8</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="1" t="s">
         <v>158</v>
       </c>
       <c r="D30">
         <v>2</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F30" t="s">
         <v>17</v>
       </c>
-      <c r="G30" s="6" t="s">
+      <c r="G30" s="4" t="s">
         <v>165</v>
       </c>
       <c r="H30" t="s">
         <v>17</v>
       </c>
-      <c r="I30" s="6" t="s">
+      <c r="I30" s="4" t="s">
         <v>166</v>
       </c>
       <c r="J30" t="s">
         <v>17</v>
       </c>
-      <c r="K30" s="6" t="s">
+      <c r="K30" s="4" t="s">
         <v>167</v>
       </c>
       <c r="L30" t="s">
         <v>17</v>
       </c>
-      <c r="M30" s="6" t="s">
+      <c r="M30" s="4" t="s">
         <v>168</v>
       </c>
       <c r="N30" t="s">
@@ -3379,13 +3313,13 @@
       <c r="B31">
         <v>8</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="1" t="s">
         <v>158</v>
       </c>
       <c r="D31">
         <v>3</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="4" t="s">
         <v>169</v>
       </c>
       <c r="F31" t="s">
@@ -3397,7 +3331,7 @@
       <c r="H31" t="s">
         <v>17</v>
       </c>
-      <c r="I31" s="6" t="s">
+      <c r="I31" s="4" t="s">
         <v>171</v>
       </c>
       <c r="J31" t="s">
@@ -3409,7 +3343,7 @@
       <c r="L31" t="s">
         <v>17</v>
       </c>
-      <c r="M31" s="6" t="s">
+      <c r="M31" s="4" t="s">
         <v>173</v>
       </c>
       <c r="N31" t="s">
@@ -3423,37 +3357,37 @@
       <c r="B32">
         <v>8</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="1" t="s">
         <v>158</v>
       </c>
       <c r="D32">
         <v>4</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="4" t="s">
         <v>174</v>
       </c>
       <c r="F32" t="s">
         <v>17</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="4" t="s">
         <v>175</v>
       </c>
       <c r="H32" t="s">
         <v>17</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I32" s="4" t="s">
         <v>176</v>
       </c>
       <c r="J32" t="s">
         <v>17</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" s="4" t="s">
         <v>177</v>
       </c>
       <c r="L32" t="s">
         <v>17</v>
       </c>
-      <c r="M32" s="6" t="s">
+      <c r="M32" s="4" t="s">
         <v>178</v>
       </c>
       <c r="N32" t="s">
@@ -3467,13 +3401,13 @@
       <c r="B33">
         <v>8</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="1" t="s">
         <v>158</v>
       </c>
       <c r="D33">
         <v>5</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="4" t="s">
         <v>179</v>
       </c>
       <c r="F33" t="s">
@@ -3485,7 +3419,7 @@
       <c r="H33" t="s">
         <v>17</v>
       </c>
-      <c r="I33" s="6" t="s">
+      <c r="I33" s="4" t="s">
         <v>181</v>
       </c>
       <c r="J33" t="s">
@@ -3497,71 +3431,71 @@
       <c r="L33" t="s">
         <v>17</v>
       </c>
-      <c r="M33" s="6" t="s">
+      <c r="M33" s="4" t="s">
         <v>183</v>
       </c>
       <c r="N33" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="34" ht="409.5" spans="1:14">
+    <row r="34" ht="247" spans="1:14">
       <c r="A34" t="s">
         <v>14</v>
       </c>
       <c r="B34">
         <v>9</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="1" t="s">
         <v>184</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="4" t="s">
         <v>185</v>
       </c>
       <c r="F34" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="6" t="s">
+      <c r="G34" s="4" t="s">
         <v>186</v>
       </c>
       <c r="H34" t="s">
         <v>17</v>
       </c>
-      <c r="I34" s="6" t="s">
+      <c r="I34" s="4" t="s">
         <v>187</v>
       </c>
       <c r="J34" t="s">
         <v>17</v>
       </c>
-      <c r="K34" s="6" t="s">
+      <c r="K34" s="4" t="s">
         <v>188</v>
       </c>
       <c r="L34" t="s">
         <v>17</v>
       </c>
-      <c r="M34" s="6" t="s">
+      <c r="M34" s="4" t="s">
         <v>189</v>
       </c>
       <c r="N34" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="35" ht="409.5" spans="1:14">
+    <row r="35" ht="370" spans="1:14">
       <c r="A35" t="s">
         <v>14</v>
       </c>
       <c r="B35">
         <v>9</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="1" t="s">
         <v>184</v>
       </c>
       <c r="D35">
         <v>2</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="4" t="s">
         <v>190</v>
       </c>
       <c r="F35" t="s">
@@ -3573,7 +3507,7 @@
       <c r="H35" t="s">
         <v>17</v>
       </c>
-      <c r="I35" s="6" t="s">
+      <c r="I35" s="4" t="s">
         <v>192</v>
       </c>
       <c r="J35" t="s">
@@ -3582,7 +3516,7 @@
       <c r="L35" t="s">
         <v>17</v>
       </c>
-      <c r="M35" s="6" t="s">
+      <c r="M35" s="4" t="s">
         <v>193</v>
       </c>
       <c r="N35" t="s">
@@ -3596,37 +3530,37 @@
       <c r="B36">
         <v>9</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="1" t="s">
         <v>184</v>
       </c>
       <c r="D36">
         <v>3</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="4" t="s">
         <v>194</v>
       </c>
       <c r="F36" t="s">
         <v>17</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="G36" s="4" t="s">
         <v>195</v>
       </c>
       <c r="H36" t="s">
         <v>17</v>
       </c>
-      <c r="I36" s="6" t="s">
+      <c r="I36" s="4" t="s">
         <v>196</v>
       </c>
       <c r="J36" t="s">
         <v>17</v>
       </c>
-      <c r="K36" s="6" t="s">
+      <c r="K36" s="4" t="s">
         <v>197</v>
       </c>
       <c r="L36" t="s">
         <v>17</v>
       </c>
-      <c r="M36" s="6" t="s">
+      <c r="M36" s="4" t="s">
         <v>198</v>
       </c>
       <c r="N36" t="s">
@@ -3640,13 +3574,13 @@
       <c r="B37">
         <v>10</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="1" t="s">
         <v>199</v>
       </c>
       <c r="D37">
         <v>1</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="4" t="s">
         <v>200</v>
       </c>
       <c r="F37">
@@ -3658,7 +3592,7 @@
       <c r="H37" t="s">
         <v>17</v>
       </c>
-      <c r="I37" s="6" t="s">
+      <c r="I37" s="4" t="s">
         <v>202</v>
       </c>
       <c r="J37" t="s">
@@ -3670,7 +3604,7 @@
       <c r="L37" t="s">
         <v>17</v>
       </c>
-      <c r="M37" s="6" t="s">
+      <c r="M37" s="4" t="s">
         <v>204</v>
       </c>
       <c r="N37" t="s">
@@ -3684,37 +3618,37 @@
       <c r="B38">
         <v>10</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="1" t="s">
         <v>199</v>
       </c>
       <c r="D38">
         <v>2</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E38" s="4" t="s">
         <v>205</v>
       </c>
       <c r="F38" t="s">
         <v>17</v>
       </c>
-      <c r="G38" s="6" t="s">
+      <c r="G38" s="4" t="s">
         <v>206</v>
       </c>
       <c r="H38" t="s">
         <v>17</v>
       </c>
-      <c r="I38" s="6" t="s">
+      <c r="I38" s="4" t="s">
         <v>207</v>
       </c>
       <c r="J38" t="s">
         <v>17</v>
       </c>
-      <c r="K38" s="6" t="s">
+      <c r="K38" s="4" t="s">
         <v>208</v>
       </c>
       <c r="L38" t="s">
         <v>17</v>
       </c>
-      <c r="M38" s="6" t="s">
+      <c r="M38" s="4" t="s">
         <v>209</v>
       </c>
       <c r="N38" t="s">
@@ -3728,13 +3662,13 @@
       <c r="B39">
         <v>10</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="1" t="s">
         <v>199</v>
       </c>
       <c r="D39">
         <v>3</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="E39" s="4" t="s">
         <v>210</v>
       </c>
       <c r="F39" t="s">
@@ -3746,7 +3680,7 @@
       <c r="H39" t="s">
         <v>17</v>
       </c>
-      <c r="I39" s="6" t="s">
+      <c r="I39" s="4" t="s">
         <v>212</v>
       </c>
       <c r="J39" t="s">
@@ -3758,7 +3692,7 @@
       <c r="L39" t="s">
         <v>17</v>
       </c>
-      <c r="M39" s="6" t="s">
+      <c r="M39" s="4" t="s">
         <v>214</v>
       </c>
       <c r="N39" t="s">
@@ -3772,37 +3706,37 @@
       <c r="B40">
         <v>10</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="1" t="s">
         <v>199</v>
       </c>
       <c r="D40">
         <v>4</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="E40" s="4" t="s">
         <v>215</v>
       </c>
       <c r="F40" t="s">
         <v>17</v>
       </c>
-      <c r="G40" s="6" t="s">
+      <c r="G40" s="4" t="s">
         <v>216</v>
       </c>
       <c r="H40" t="s">
         <v>17</v>
       </c>
-      <c r="I40" s="6" t="s">
+      <c r="I40" s="4" t="s">
         <v>217</v>
       </c>
       <c r="J40" t="s">
         <v>17</v>
       </c>
-      <c r="K40" s="6" t="s">
+      <c r="K40" s="4" t="s">
         <v>218</v>
       </c>
       <c r="L40" t="s">
         <v>17</v>
       </c>
-      <c r="M40" s="6" t="s">
+      <c r="M40" s="4" t="s">
         <v>219</v>
       </c>
       <c r="N40" t="s">
@@ -3816,13 +3750,13 @@
       <c r="B41">
         <v>11</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="1" t="s">
         <v>220</v>
       </c>
       <c r="D41">
         <v>1</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="E41" s="4" t="s">
         <v>221</v>
       </c>
       <c r="F41">
@@ -3834,7 +3768,7 @@
       <c r="H41">
         <v>4</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="I41" s="4" t="s">
         <v>223</v>
       </c>
       <c r="J41">
@@ -3846,7 +3780,7 @@
       <c r="L41">
         <v>5</v>
       </c>
-      <c r="M41" s="6" t="s">
+      <c r="M41" s="4" t="s">
         <v>225</v>
       </c>
       <c r="N41">
@@ -3860,37 +3794,37 @@
       <c r="B42">
         <v>11</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="1" t="s">
         <v>220</v>
       </c>
       <c r="D42">
         <v>2</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="E42" s="4" t="s">
         <v>226</v>
       </c>
       <c r="F42" t="s">
         <v>17</v>
       </c>
-      <c r="G42" s="6" t="s">
+      <c r="G42" s="4" t="s">
         <v>227</v>
       </c>
       <c r="H42" t="s">
         <v>17</v>
       </c>
-      <c r="I42" s="6" t="s">
+      <c r="I42" s="4" t="s">
         <v>228</v>
       </c>
       <c r="J42" t="s">
         <v>17</v>
       </c>
-      <c r="K42" s="6" t="s">
+      <c r="K42" s="4" t="s">
         <v>229</v>
       </c>
       <c r="L42" t="s">
         <v>17</v>
       </c>
-      <c r="M42" s="6" t="s">
+      <c r="M42" s="4" t="s">
         <v>230</v>
       </c>
       <c r="N42" t="s">
@@ -3904,13 +3838,13 @@
       <c r="B43">
         <v>11</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="1" t="s">
         <v>220</v>
       </c>
       <c r="D43">
         <v>3</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="E43" s="4" t="s">
         <v>231</v>
       </c>
       <c r="F43" t="s">
@@ -3922,7 +3856,7 @@
       <c r="H43" t="s">
         <v>17</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="I43" s="4" t="s">
         <v>233</v>
       </c>
       <c r="J43" t="s">
@@ -3934,7 +3868,7 @@
       <c r="L43" t="s">
         <v>17</v>
       </c>
-      <c r="M43" s="6" t="s">
+      <c r="M43" s="4" t="s">
         <v>235</v>
       </c>
       <c r="N43" t="s">
@@ -3948,44 +3882,44 @@
       <c r="B44">
         <v>11</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="1" t="s">
         <v>220</v>
       </c>
       <c r="D44">
         <v>4</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="E44" s="4" t="s">
         <v>236</v>
       </c>
       <c r="F44" t="s">
         <v>17</v>
       </c>
-      <c r="G44" s="6" t="s">
+      <c r="G44" s="4" t="s">
         <v>237</v>
       </c>
       <c r="H44" t="s">
         <v>17</v>
       </c>
-      <c r="I44" s="6" t="s">
+      <c r="I44" s="4" t="s">
         <v>238</v>
       </c>
       <c r="J44" t="s">
         <v>17</v>
       </c>
-      <c r="K44" s="6" t="s">
+      <c r="K44" s="4" t="s">
         <v>239</v>
       </c>
       <c r="L44" t="s">
         <v>17</v>
       </c>
-      <c r="M44" s="6" t="s">
+      <c r="M44" s="4" t="s">
         <v>240</v>
       </c>
       <c r="N44" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="45" ht="335" spans="1:14">
+    <row r="45" ht="300" spans="1:14">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -3998,7 +3932,7 @@
       <c r="D45">
         <v>1</v>
       </c>
-      <c r="E45" s="6" t="s">
+      <c r="E45" s="4" t="s">
         <v>242</v>
       </c>
       <c r="F45" t="s">
@@ -4010,7 +3944,7 @@
       <c r="H45" t="s">
         <v>17</v>
       </c>
-      <c r="I45" s="6" t="s">
+      <c r="I45" s="4" t="s">
         <v>244</v>
       </c>
       <c r="J45" t="s">
@@ -4022,7 +3956,7 @@
       <c r="L45" t="s">
         <v>17</v>
       </c>
-      <c r="M45" s="6" t="s">
+      <c r="M45" s="4" t="s">
         <v>246</v>
       </c>
       <c r="N45" t="s">
@@ -4036,37 +3970,37 @@
       <c r="B46">
         <v>12</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="1" t="s">
         <v>241</v>
       </c>
       <c r="D46">
         <v>2</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="E46" s="4" t="s">
         <v>247</v>
       </c>
       <c r="F46" t="s">
         <v>17</v>
       </c>
-      <c r="G46" s="6" t="s">
+      <c r="G46" s="4" t="s">
         <v>248</v>
       </c>
       <c r="H46" t="s">
         <v>17</v>
       </c>
-      <c r="I46" s="6" t="s">
+      <c r="I46" s="4" t="s">
         <v>249</v>
       </c>
       <c r="J46" t="s">
         <v>17</v>
       </c>
-      <c r="K46" s="6" t="s">
+      <c r="K46" s="4" t="s">
         <v>250</v>
       </c>
       <c r="L46" t="s">
         <v>17</v>
       </c>
-      <c r="M46" s="6" t="s">
+      <c r="M46" s="4" t="s">
         <v>251</v>
       </c>
       <c r="N46" t="s">
@@ -4080,13 +4014,13 @@
       <c r="B47">
         <v>12</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="1" t="s">
         <v>241</v>
       </c>
       <c r="D47">
         <v>3</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="E47" s="4" t="s">
         <v>252</v>
       </c>
       <c r="F47" t="s">
@@ -4098,19 +4032,19 @@
       <c r="H47" t="s">
         <v>17</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="I47" s="4" t="s">
         <v>254</v>
       </c>
       <c r="J47" t="s">
         <v>17</v>
       </c>
-      <c r="K47" s="6" t="s">
+      <c r="K47" s="4" t="s">
         <v>255</v>
       </c>
       <c r="L47" t="s">
         <v>17</v>
       </c>
-      <c r="M47" s="6" t="s">
+      <c r="M47" s="4" t="s">
         <v>256</v>
       </c>
       <c r="N47" t="s">
@@ -4124,37 +4058,37 @@
       <c r="B48">
         <v>12</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="1" t="s">
         <v>241</v>
       </c>
       <c r="D48">
         <v>4</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="E48" s="4" t="s">
         <v>257</v>
       </c>
       <c r="F48" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="6" t="s">
+      <c r="G48" s="4" t="s">
         <v>258</v>
       </c>
       <c r="H48" t="s">
         <v>17</v>
       </c>
-      <c r="I48" s="6" t="s">
+      <c r="I48" s="4" t="s">
         <v>259</v>
       </c>
       <c r="J48" t="s">
         <v>17</v>
       </c>
-      <c r="K48" s="6" t="s">
+      <c r="K48" s="4" t="s">
         <v>260</v>
       </c>
       <c r="L48" t="s">
         <v>17</v>
       </c>
-      <c r="M48" s="6" t="s">
+      <c r="M48" s="4" t="s">
         <v>261</v>
       </c>
       <c r="N48" t="s">
@@ -4165,66 +4099,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="17.6" outlineLevelRow="2" outlineLevelCol="5"/>
-  <cols>
-    <col min="1" max="2" width="8.88888888888889" style="1"/>
-    <col min="3" max="3" width="44.5555555555556" style="1" customWidth="1"/>
-    <col min="4" max="4" width="38.5416666666667" style="1" customWidth="1"/>
-    <col min="5" max="5" width="37.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.2638888888889" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.88888888888889" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="2" ht="159" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="3" ht="106" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>